<commit_message>
used: lp register Rodrigo
</commit_message>
<xml_diff>
--- a/98 - Excels/LP-Register.xlsx
+++ b/98 - Excels/LP-Register.xlsx
@@ -568,7 +568,11 @@
           <t>Cadastrada</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -631,7 +635,11 @@
           <t>Cadastrada</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr"/>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -696,7 +704,11 @@
           <t>Cadastrada</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr"/>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -759,7 +771,11 @@
           <t>Cadastrada</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr"/>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -822,7 +838,11 @@
           <t>Cadastrada</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr"/>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -885,7 +905,11 @@
           <t>Cadastrada</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr"/>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -948,7 +972,11 @@
           <t>Cadastrada</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr"/>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1011,7 +1039,11 @@
           <t>Cadastrada</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr"/>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1074,7 +1106,11 @@
           <t>Cadastrada</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr"/>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1139,7 +1175,11 @@
           <t>Cadastrada</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr"/>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1202,7 +1242,11 @@
           <t>Cadastrada</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr"/>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1265,7 +1309,11 @@
           <t>Cadastrada</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr"/>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1328,7 +1376,11 @@
           <t>Cadastrada</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr"/>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1391,7 +1443,11 @@
           <t>Cadastrada</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr"/>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1454,7 +1510,11 @@
           <t>Cadastrada</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr"/>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1517,7 +1577,11 @@
           <t>Cadastrada</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr"/>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1580,7 +1644,11 @@
           <t>Cadastrada</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr"/>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1643,7 +1711,11 @@
           <t>Cadastrada</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr"/>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1708,7 +1780,11 @@
           <t>Cadastrada</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr"/>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1771,7 +1847,11 @@
           <t>Cadastrada</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr"/>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1834,7 +1914,11 @@
           <t>Cadastrada</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr"/>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1897,7 +1981,11 @@
           <t>Cadastrada</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr"/>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1960,7 +2048,11 @@
           <t>Cadastrada</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr"/>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -9953,7 +10045,11 @@
           <t>LP-057115</t>
         </is>
       </c>
-      <c r="N150" t="inlineStr"/>
+      <c r="N150" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
       <c r="O150" t="inlineStr"/>
     </row>
     <row r="151">
@@ -10012,7 +10108,11 @@
           <t>LP-057114</t>
         </is>
       </c>
-      <c r="N151" t="inlineStr"/>
+      <c r="N151" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
       <c r="O151" t="inlineStr"/>
     </row>
     <row r="152">
@@ -10071,7 +10171,11 @@
           <t>LP-057142</t>
         </is>
       </c>
-      <c r="N152" t="inlineStr"/>
+      <c r="N152" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
       <c r="O152" t="inlineStr"/>
     </row>
     <row r="153">
@@ -10130,7 +10234,11 @@
           <t>LP-057141</t>
         </is>
       </c>
-      <c r="N153" t="inlineStr"/>
+      <c r="N153" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
       <c r="O153" t="inlineStr"/>
     </row>
     <row r="154">
@@ -10189,7 +10297,11 @@
           <t>LP-057140</t>
         </is>
       </c>
-      <c r="N154" t="inlineStr"/>
+      <c r="N154" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
       <c r="O154" t="inlineStr"/>
     </row>
     <row r="155">
@@ -10248,7 +10360,11 @@
           <t>LP-057137</t>
         </is>
       </c>
-      <c r="N155" t="inlineStr"/>
+      <c r="N155" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
       <c r="O155" t="inlineStr"/>
     </row>
     <row r="156">
@@ -10307,7 +10423,11 @@
           <t>LP-057134</t>
         </is>
       </c>
-      <c r="N156" t="inlineStr"/>
+      <c r="N156" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
       <c r="O156" t="inlineStr"/>
     </row>
     <row r="157">
@@ -10368,7 +10488,11 @@
           <t>LP-057133</t>
         </is>
       </c>
-      <c r="N157" t="inlineStr"/>
+      <c r="N157" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
       <c r="O157" t="inlineStr"/>
     </row>
     <row r="158">
@@ -10427,7 +10551,11 @@
           <t>LP-057132</t>
         </is>
       </c>
-      <c r="N158" t="inlineStr"/>
+      <c r="N158" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
       <c r="O158" t="inlineStr"/>
     </row>
     <row r="159">
@@ -10486,7 +10614,11 @@
           <t>LP-057128</t>
         </is>
       </c>
-      <c r="N159" t="inlineStr"/>
+      <c r="N159" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
       <c r="O159" t="inlineStr"/>
     </row>
     <row r="160">
@@ -10547,7 +10679,11 @@
           <t>LP-057130</t>
         </is>
       </c>
-      <c r="N160" t="inlineStr"/>
+      <c r="N160" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
       <c r="O160" t="inlineStr"/>
     </row>
     <row r="161">
@@ -10608,7 +10744,11 @@
           <t>LP-057129</t>
         </is>
       </c>
-      <c r="N161" t="inlineStr"/>
+      <c r="N161" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
       <c r="O161" t="inlineStr"/>
     </row>
     <row r="162">
@@ -10669,7 +10809,11 @@
           <t>LP-057126</t>
         </is>
       </c>
-      <c r="N162" t="inlineStr"/>
+      <c r="N162" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
       <c r="O162" t="inlineStr"/>
     </row>
     <row r="163">
@@ -10728,7 +10872,11 @@
           <t>LP-057125</t>
         </is>
       </c>
-      <c r="N163" t="inlineStr"/>
+      <c r="N163" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
       <c r="O163" t="inlineStr"/>
     </row>
     <row r="164">
@@ -10789,7 +10937,11 @@
           <t>LP-057164</t>
         </is>
       </c>
-      <c r="N164" t="inlineStr"/>
+      <c r="N164" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
       <c r="O164" t="inlineStr"/>
     </row>
     <row r="165">
@@ -10848,7 +11000,11 @@
           <t>LP-057047</t>
         </is>
       </c>
-      <c r="N165" t="inlineStr"/>
+      <c r="N165" t="inlineStr">
+        <is>
+          <t>Cadastrada</t>
+        </is>
+      </c>
       <c r="O165" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>